<commit_message>
added fuzzy searching in emacs and 1 index in tmux
</commit_message>
<xml_diff>
--- a/emacs_cheatsheet.xlsx
+++ b/emacs_cheatsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kanishk/professional/configs/configs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD730E29-31E0-3941-9BB1-1685ABE1347E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1C727A-F33F-8749-867B-68D4ADB0C99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="680" windowWidth="25820" windowHeight="18960" xr2:uid="{DB0BB786-CC79-3246-8EE5-25725AD88A98}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{DB0BB786-CC79-3246-8EE5-25725AD88A98}"/>
   </bookViews>
   <sheets>
     <sheet name="emacs_cheatsheet" sheetId="1" r:id="rId1"/>
@@ -1416,7 +1416,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
added ruff's fix issues on save
</commit_message>
<xml_diff>
--- a/emacs_cheatsheet.xlsx
+++ b/emacs_cheatsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kanishk/professional/configs/configs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1C727A-F33F-8749-867B-68D4ADB0C99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC22DF6-72C7-D34B-BF29-2F50629103B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{DB0BB786-CC79-3246-8EE5-25725AD88A98}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="137">
   <si>
     <t>Command</t>
   </si>
@@ -407,6 +407,30 @@
   </si>
   <si>
     <t>go to previous mark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">             </t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>diff range</t>
+  </si>
+  <si>
+    <t>ediff of range</t>
+  </si>
+  <si>
+    <t>diff options</t>
+  </si>
+  <si>
+    <t>magit-cherry</t>
+  </si>
+  <si>
+    <t>see commets diff</t>
   </si>
 </sst>
 </file>
@@ -1274,7 +1298,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEC42473-9417-564E-94BB-C46BAE2BE950}">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
@@ -1416,7 +1440,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="B13" t="s">
         <v>24</v>
@@ -1865,50 +1889,94 @@
         <v>116</v>
       </c>
     </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>92</v>
+      </c>
+      <c r="B56" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" t="s">
+        <v>134</v>
+      </c>
+    </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C57" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="C58" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" ht="19" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>124</v>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>92</v>
+      </c>
+      <c r="B59" t="s">
+        <v>135</v>
+      </c>
+      <c r="C59" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>125</v>
+        <v>117</v>
+      </c>
+      <c r="B63" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
+        <v>117</v>
+      </c>
+      <c r="B64" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="19" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added better alias for emacsclient
</commit_message>
<xml_diff>
--- a/emacs_cheatsheet.xlsx
+++ b/emacs_cheatsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kanishk/professional/configs/configs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC22DF6-72C7-D34B-BF29-2F50629103B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AA37FC-7BD4-0A4C-85BA-995231346208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{DB0BB786-CC79-3246-8EE5-25725AD88A98}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="138">
   <si>
     <t>Command</t>
   </si>
@@ -431,6 +431,9 @@
   </si>
   <si>
     <t>see commets diff</t>
+  </si>
+  <si>
+    <t>flycheck list errors</t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEC42473-9417-564E-94BB-C46BAE2BE950}">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
@@ -1980,6 +1983,11 @@
         <v>126</v>
       </c>
     </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>